<commit_message>
prutsen, excel duidelijker met cefr voor controle
</commit_message>
<xml_diff>
--- a/ruwe_data/Duitse taalvaardigheid onderzoek(1-154).csv.xlsx
+++ b/ruwe_data/Duitse taalvaardigheid onderzoek(1-154).csv.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jesse\Desktop\wetenschappelijke_cyclus_onderzoek\ruwe_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DBF42AA2-AA4E-4FAF-A35B-B147AC2F5C95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24ACDC14-2CD1-4E78-BD4B-4760E5024DC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9665" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9705" uniqueCount="343">
   <si>
     <t>ID</t>
   </si>
@@ -1055,15 +1055,27 @@
   <si>
     <t>ANSWERS</t>
   </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>B1</t>
+  </si>
+  <si>
+    <t>B2</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="m/d/yy\ h:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm:ss"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1075,6 +1087,12 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1158,22 +1176,22 @@
   </cellStyleXfs>
   <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1191,16 +1209,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -32683,7 +32691,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAA902A0-895F-418A-837D-6B13AF9633CC}">
-  <dimension ref="A2:BN156"/>
+  <dimension ref="A1:BN156"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2.36328125" bestFit="1" customWidth="1"/>
@@ -32753,6 +32761,128 @@
     <col min="66" max="66" width="53.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:66" x14ac:dyDescent="0.35">
+      <c r="Q1" t="s">
+        <v>339</v>
+      </c>
+      <c r="R1" t="s">
+        <v>339</v>
+      </c>
+      <c r="S1" t="s">
+        <v>339</v>
+      </c>
+      <c r="T1" t="s">
+        <v>339</v>
+      </c>
+      <c r="U1" t="s">
+        <v>339</v>
+      </c>
+      <c r="V1" t="s">
+        <v>339</v>
+      </c>
+      <c r="W1" t="s">
+        <v>339</v>
+      </c>
+      <c r="X1" t="s">
+        <v>339</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>339</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>339</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>340</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>340</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>340</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>340</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>340</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>340</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>340</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>340</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>340</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>340</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>341</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>341</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>341</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>341</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>341</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>341</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>341</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>341</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>341</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>341</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>342</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>342</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>342</v>
+      </c>
+      <c r="AX1" t="s">
+        <v>342</v>
+      </c>
+      <c r="AY1" t="s">
+        <v>342</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>342</v>
+      </c>
+      <c r="BA1" t="s">
+        <v>342</v>
+      </c>
+      <c r="BB1" t="s">
+        <v>342</v>
+      </c>
+      <c r="BC1" t="s">
+        <v>342</v>
+      </c>
+      <c r="BD1" t="s">
+        <v>342</v>
+      </c>
+    </row>
     <row r="2" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A2" t="str">
         <f>(TRIM(LOWER(Sheet1!A2)))</f>
@@ -73984,12 +74114,13 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="Q3:BN156">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>0</formula>
+    </cfRule>
     <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
-      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>